<commit_message>
[DONE]: Project finalized; Enhanced node-red and knime flows; Added relative paths; Improved regex rules; node-red and knime connection created by GUI
</commit_message>
<xml_diff>
--- a/knime/etl_food_stock/data/pipeline-execution-review/pipeline_execution_review.xlsx
+++ b/knime/etl_food_stock/data/pipeline-execution-review/pipeline_execution_review.xlsx
@@ -56,7 +56,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -97,23 +97,23 @@
       </c>
       <c r="H1" t="inlineStr" s="0">
         <is>
-          <t>expirationdate</t>
+          <t>expiration_date</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="0">
         <is>
-          <t>Maca Riscadinha</t>
+          <t>Pão</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t>Fruits</t>
+          <t>Padaria</t>
         </is>
       </c>
       <c r="C2" t="n" s="0">
-        <v>45.5</v>
+        <v>15.0</v>
       </c>
       <c r="D2" s="0"/>
       <c r="E2" s="0"/>
@@ -124,140 +124,40 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="0">
         <is>
-          <t>alface frisada</t>
+          <t>Leite</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t>Vegetables</t>
+          <t>Leite</t>
         </is>
       </c>
       <c r="C3" t="n" s="0">
-        <v>30.0</v>
-      </c>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="0">
-        <is>
-          <t>PAO DE MISTURA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="0">
-        <is>
-          <t>Bakery</t>
-        </is>
-      </c>
-      <c r="C4" t="n" s="0">
-        <v>120.0</v>
-      </c>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr" s="0">
-        <is>
-          <t>Banana da Madeira</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr" s="0">
-        <is>
-          <t>Fruits</t>
-        </is>
-      </c>
-      <c r="C5" t="n" s="0">
-        <v>60.0</v>
-      </c>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr" s="0">
-        <is>
-          <t>Leite</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr" s="0">
-        <is>
-          <t>Leites meio gordo, Leites UHT</t>
-        </is>
-      </c>
-      <c r="C6" t="n" s="0">
-        <v>23.0</v>
-      </c>
-      <c r="D6" t="inlineStr" s="0">
+        <v>24.0</v>
+      </c>
+      <c r="D3" t="inlineStr" s="0">
         <is>
           <t>5601049132995</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="0">
+      <c r="E3" t="inlineStr" s="0">
         <is>
           <t>1000ml</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="0">
+      <c r="F3" t="inlineStr" s="0">
         <is>
           <t>leite</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="0">
+      <c r="G3" t="inlineStr" s="0">
         <is>
           <t>https://images.openfoodfacts.org/images/products/560/104/913/2995/front_pt.85.400.jpg</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr" s="0">
-        <is>
-          <t>02/12/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr" s="0">
-        <is>
-          <t>Leite</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr" s="0">
-        <is>
-          <t>Leites meio gordo, Leites UHT</t>
-        </is>
-      </c>
-      <c r="C7" t="n" s="0">
-        <v>120.0</v>
-      </c>
-      <c r="D7" t="inlineStr" s="0">
-        <is>
-          <t>5601049132995</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr" s="0">
-        <is>
-          <t>1000ml</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr" s="0">
-        <is>
-          <t>leite</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr" s="0">
-        <is>
-          <t>https://images.openfoodfacts.org/images/products/560/104/913/2995/front_pt.85.400.jpg</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr" s="0">
-        <is>
-          <t>27/03/2027</t>
+      <c r="H3" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -269,7 +169,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -288,21 +188,9 @@
           <t>failure_reason</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>8410500028794</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Product Matching</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>EAN not found in CSV</t>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>expiration_date</t>
         </is>
       </c>
     </row>

</xml_diff>